<commit_message>
Require whole calendar years in inputs
</commit_message>
<xml_diff>
--- a/inst/extdata/imurun_example.xlsx
+++ b/inst/extdata/imurun_example.xlsx
@@ -556,7 +556,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Observation Year  timing of the observation</t>
+          <t xml:space="preserve">  Observation Year  calendar year of the observation (1000-9999)</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Target Year       timing of the target snapshot to predict</t>
+          <t xml:space="preserve">  Target Year       calendar year of the target snapshot (1000-9999)</t>
         </is>
       </c>
     </row>

</xml_diff>